<commit_message>
Finaliza motor de conferência de folha
</commit_message>
<xml_diff>
--- a/scripts/conferencia-folha/output/resultado_conferencia_05-2026.xlsx
+++ b/scripts/conferencia-folha/output/resultado_conferencia_05-2026.xlsx
@@ -7,7 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RESUMO_GERAL" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RESUMO_TIPO_ERRO" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="RESUMO_POR_ABA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ERROS_DETALHADOS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,6 +416,286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>INDICADOR</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Competência analisada</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Linhas na prévia</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>19804</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lançamentos FOPAG</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5988</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Colaboradores em férias</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Colaboradores desligados</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total de divergências</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>966</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TIPO_ERRO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PAGO_NAO_ENVIADO</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ENVIADO_NAO_PAGO(FERIAS)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ENVIADO_NAO_PAGO</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ABA_FOPAG</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ATRASOS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADC NOT</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FALTAS</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EXTRAS</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GRAT CTI ESP</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GRAT PLT</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GRAT ROT</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GRAT FDS</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GRAT DIF PROV</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I967"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -466,7 +749,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -504,7 +787,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -597,7 +880,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -633,7 +916,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1869,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1624,7 +1907,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2387,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2142,14 +2425,14 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2187,14 +2470,14 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2232,14 +2515,14 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2277,14 +2560,14 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2322,14 +2605,14 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2367,14 +2650,14 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2412,7 +2695,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2792,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2547,14 +2830,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2592,14 +2875,14 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2635,14 +2918,14 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2680,14 +2963,14 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2725,14 +3008,14 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2770,14 +3053,14 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2815,7 +3098,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -2865,7 +3148,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2901,7 +3184,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -2953,7 +3236,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2991,7 +3274,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4319,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4072,14 +4355,14 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4117,14 +4400,14 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4162,7 +4445,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -4470,7 +4753,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4508,14 +4791,14 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4551,7 +4834,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5400,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5153,7 +5436,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5658,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5411,7 +5694,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5787,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5542,7 +5825,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -5893,7 +6176,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5929,14 +6212,14 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -5972,7 +6255,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -6413,7 +6696,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6451,7 +6734,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -6847,7 +7130,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -6885,7 +7168,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -7410,7 +7693,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -7448,7 +7731,7 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -8837,7 +9120,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -8875,7 +9158,7 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -8968,7 +9251,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -9006,7 +9289,7 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -9443,7 +9726,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -9481,14 +9764,14 @@
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -9526,14 +9809,14 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -9571,14 +9854,14 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -9616,7 +9899,7 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -9924,7 +10207,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -9962,14 +10245,14 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -10005,14 +10288,14 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -10050,7 +10333,7 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -10143,7 +10426,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -10181,14 +10464,14 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -10226,7 +10509,7 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -10538,7 +10821,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -10576,14 +10859,14 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -10621,14 +10904,14 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -10666,14 +10949,14 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -10711,7 +10994,7 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -10761,7 +11044,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -10797,14 +11080,14 @@
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -10842,7 +11125,7 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -11412,7 +11695,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -11450,14 +11733,14 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -11495,14 +11778,14 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -11540,14 +11823,14 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -11585,14 +11868,14 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -11630,14 +11913,14 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -11675,14 +11958,14 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -11720,7 +12003,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -13232,7 +13515,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -13268,7 +13551,7 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -13920,7 +14203,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -13958,14 +14241,14 @@
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -14003,14 +14286,14 @@
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -14048,14 +14331,14 @@
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -14093,14 +14376,14 @@
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -14138,7 +14421,7 @@
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -14929,7 +15212,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -14967,7 +15250,7 @@
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -16282,7 +16565,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -16320,7 +16603,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -17283,7 +17566,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -17319,7 +17602,7 @@
       </c>
       <c r="I389" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -17627,7 +17910,7 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
@@ -17663,14 +17946,14 @@
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -17706,14 +17989,14 @@
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -17749,14 +18032,14 @@
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -17792,14 +18075,14 @@
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
@@ -17835,7 +18118,7 @@
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -17885,7 +18168,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -17921,7 +18204,7 @@
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -18628,7 +18911,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -18664,7 +18947,7 @@
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -18757,7 +19040,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
@@ -18795,14 +19078,14 @@
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
@@ -18840,14 +19123,14 @@
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
@@ -18885,7 +19168,7 @@
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -19977,7 +20260,7 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
@@ -20013,14 +20296,14 @@
       </c>
       <c r="I451" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
@@ -20056,7 +20339,7 @@
       </c>
       <c r="I452" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -20407,7 +20690,7 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
@@ -20443,14 +20726,14 @@
       </c>
       <c r="I461" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
@@ -20486,7 +20769,7 @@
       </c>
       <c r="I462" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -20536,7 +20819,7 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
@@ -20572,14 +20855,14 @@
       </c>
       <c r="I464" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
@@ -20615,14 +20898,14 @@
       </c>
       <c r="I465" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
@@ -20660,7 +20943,7 @@
       </c>
       <c r="I466" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -20710,7 +20993,7 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
@@ -20746,7 +21029,7 @@
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -20882,7 +21165,7 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
@@ -20918,14 +21201,14 @@
       </c>
       <c r="I472" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
@@ -20961,14 +21244,14 @@
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
@@ -21004,7 +21287,7 @@
       </c>
       <c r="I474" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>
@@ -22468,7 +22751,7 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>MATRICULA_NAO_CONSTA_NA_PREVIA</t>
+          <t>MATRICULA_NAO_CONSTA_NA_PREVIA(DESLIGADO)</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
@@ -22500,7 +22783,7 @@
       </c>
       <c r="I510" t="inlineStr">
         <is>
-          <t>Matrícula enviada na FOPAG, mas não existe na prévia da sede.</t>
+          <t>Matrícula enviada, mas colaborador consta como desligado.</t>
         </is>
       </c>
     </row>

</xml_diff>